<commit_message>
Update project data and next steps
</commit_message>
<xml_diff>
--- a/00_Info_proporcionada/DATOS GRUPOS-2026.xlsx
+++ b/00_Info_proporcionada/DATOS GRUPOS-2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Unidades compartidas\Practicas_Inst2\4_GLPs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Unidades compartidas\Practicas_Inst2\4_GLPs\00_Info_proporcionada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01EE7A6C-A1FD-4BA1-B139-A731CFC17FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099216A6-2F2A-4F7E-B1CB-474EF9BFD740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -782,11 +782,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1184,10 +1184,10 @@
       <c r="G2" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>107</v>
       </c>
       <c r="J2" s="7" t="s">
@@ -1227,8 +1227,8 @@
         <v>208</v>
       </c>
       <c r="G3" s="11"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="13"/>
       <c r="J3" s="7" t="s">
         <v>125</v>
       </c>
@@ -1266,8 +1266,8 @@
         <v>208</v>
       </c>
       <c r="G4" s="11"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
       <c r="J4" s="7" t="s">
         <v>134</v>
       </c>
@@ -1305,8 +1305,8 @@
         <v>208</v>
       </c>
       <c r="G5" s="11"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="13"/>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
@@ -1334,10 +1334,10 @@
       <c r="G6" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="13" t="s">
         <v>108</v>
       </c>
       <c r="J6" s="7" t="s">
@@ -1377,8 +1377,8 @@
         <v>209</v>
       </c>
       <c r="G7" s="11"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="13"/>
       <c r="J7" s="7" t="s">
         <v>129</v>
       </c>
@@ -1416,8 +1416,8 @@
         <v>209</v>
       </c>
       <c r="G8" s="11"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="13"/>
       <c r="J8" s="7" t="s">
         <v>134</v>
       </c>
@@ -1455,8 +1455,8 @@
         <v>209</v>
       </c>
       <c r="G9" s="11"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
@@ -1484,10 +1484,10 @@
       <c r="G10" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="13" t="s">
         <v>109</v>
       </c>
       <c r="J10" s="7" t="s">
@@ -1527,8 +1527,8 @@
         <v>210</v>
       </c>
       <c r="G11" s="11"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="13"/>
       <c r="J11" s="7" t="s">
         <v>125</v>
       </c>
@@ -1566,8 +1566,8 @@
         <v>210</v>
       </c>
       <c r="G12" s="11"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="13"/>
       <c r="J12" s="7" t="s">
         <v>134</v>
       </c>
@@ -1605,8 +1605,8 @@
         <v>210</v>
       </c>
       <c r="G13" s="11"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="13"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -1636,10 +1636,10 @@
       <c r="G14" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="13" t="s">
         <v>110</v>
       </c>
       <c r="J14" s="7" t="s">
@@ -1679,8 +1679,8 @@
         <v>211</v>
       </c>
       <c r="G15" s="11"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="13"/>
       <c r="J15" s="7" t="s">
         <v>125</v>
       </c>
@@ -1718,8 +1718,8 @@
         <v>211</v>
       </c>
       <c r="G16" s="11"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="13"/>
       <c r="J16" s="7" t="s">
         <v>134</v>
       </c>
@@ -1757,8 +1757,8 @@
         <v>211</v>
       </c>
       <c r="G17" s="11"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="13"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -1788,10 +1788,10 @@
       <c r="G18" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I18" s="12" t="s">
+      <c r="I18" s="13" t="s">
         <v>111</v>
       </c>
       <c r="J18" s="7" t="s">
@@ -1831,8 +1831,8 @@
         <v>212</v>
       </c>
       <c r="G19" s="11"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="13"/>
       <c r="J19" s="7" t="s">
         <v>125</v>
       </c>
@@ -1870,8 +1870,8 @@
         <v>212</v>
       </c>
       <c r="G20" s="11"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="13"/>
       <c r="J20" s="7" t="s">
         <v>134</v>
       </c>
@@ -1909,8 +1909,8 @@
         <v>212</v>
       </c>
       <c r="G21" s="11"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="13"/>
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
@@ -1938,10 +1938,10 @@
       <c r="G22" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="13" t="s">
         <v>116</v>
       </c>
       <c r="J22" s="7" t="s">
@@ -1981,8 +1981,8 @@
         <v>213</v>
       </c>
       <c r="G23" s="11"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="13"/>
       <c r="J23" s="7" t="s">
         <v>125</v>
       </c>
@@ -2020,8 +2020,8 @@
         <v>213</v>
       </c>
       <c r="G24" s="11"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="13"/>
       <c r="J24" s="7" t="s">
         <v>134</v>
       </c>
@@ -2059,8 +2059,8 @@
         <v>213</v>
       </c>
       <c r="G25" s="11"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="13"/>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
@@ -2088,10 +2088,10 @@
       <c r="G26" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I26" s="12" t="s">
+      <c r="I26" s="13" t="s">
         <v>112</v>
       </c>
       <c r="J26" s="7" t="s">
@@ -2131,8 +2131,8 @@
         <v>214</v>
       </c>
       <c r="G27" s="11"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="13"/>
       <c r="J27" s="7" t="s">
         <v>125</v>
       </c>
@@ -2170,8 +2170,8 @@
         <v>214</v>
       </c>
       <c r="G28" s="11"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="13"/>
       <c r="J28" s="7" t="s">
         <v>134</v>
       </c>
@@ -2209,8 +2209,8 @@
         <v>214</v>
       </c>
       <c r="G29" s="11"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="13"/>
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
       <c r="L29" s="7"/>
@@ -2238,10 +2238,10 @@
       <c r="G30" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="H30" s="13" t="s">
+      <c r="H30" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I30" s="12" t="s">
+      <c r="I30" s="13" t="s">
         <v>113</v>
       </c>
       <c r="J30" s="7" t="s">
@@ -2281,8 +2281,8 @@
         <v>215</v>
       </c>
       <c r="G31" s="11"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="13"/>
       <c r="J31" s="7" t="s">
         <v>125</v>
       </c>
@@ -2320,8 +2320,8 @@
         <v>215</v>
       </c>
       <c r="G32" s="11"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="13"/>
       <c r="J32" s="7" t="s">
         <v>134</v>
       </c>
@@ -2359,8 +2359,8 @@
         <v>215</v>
       </c>
       <c r="G33" s="11"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="13"/>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -2388,10 +2388,10 @@
       <c r="G34" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="H34" s="13" t="s">
+      <c r="H34" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I34" s="12" t="s">
+      <c r="I34" s="13" t="s">
         <v>114</v>
       </c>
       <c r="J34" s="7" t="s">
@@ -2431,8 +2431,8 @@
         <v>216</v>
       </c>
       <c r="G35" s="11"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="13"/>
       <c r="J35" s="7" t="s">
         <v>125</v>
       </c>
@@ -2470,8 +2470,8 @@
         <v>216</v>
       </c>
       <c r="G36" s="11"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="13"/>
       <c r="J36" s="7" t="s">
         <v>134</v>
       </c>
@@ -2509,8 +2509,8 @@
         <v>216</v>
       </c>
       <c r="G37" s="11"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="13"/>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
@@ -2538,10 +2538,10 @@
       <c r="G38" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="H38" s="13" t="s">
+      <c r="H38" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I38" s="12" t="s">
+      <c r="I38" s="13" t="s">
         <v>115</v>
       </c>
       <c r="J38" s="7" t="s">
@@ -2583,8 +2583,8 @@
         <v>217</v>
       </c>
       <c r="G39" s="11"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="13"/>
       <c r="J39" s="7" t="s">
         <v>125</v>
       </c>
@@ -2608,24 +2608,6 @@
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <autoFilter ref="A1:F39" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="30">
-    <mergeCell ref="G34:G37"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="I34:I37"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="G26:G29"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="I26:I29"/>
-    <mergeCell ref="G30:G33"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="I30:I33"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="I18:I21"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="I22:I25"/>
     <mergeCell ref="G14:G17"/>
     <mergeCell ref="I14:I17"/>
     <mergeCell ref="H14:H17"/>
@@ -2638,6 +2620,24 @@
     <mergeCell ref="G10:G13"/>
     <mergeCell ref="I6:I9"/>
     <mergeCell ref="I10:I13"/>
+    <mergeCell ref="G18:G21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="I18:I21"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="I26:I29"/>
+    <mergeCell ref="G30:G33"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="I30:I33"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="I34:I37"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>

</xml_diff>